<commit_message>
Add presentation, fix Update instruction sheet
Remove the statement that filled but not updated fields are reported -
the program does not do this.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016HeHTepPuvp42QB137aYqB
</commit_message>
<xml_diff>
--- a/documents/instruction_sheets/Instructions_Update.xlsx
+++ b/documents/instruction_sheets/Instructions_Update.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -784,160 +784,152 @@
     <row r="29" ht="17" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>• Fields that are filled in the template but not updated by SAP are reported in the output.</t>
+          <t>• The material must exist for the selected material type / industry sector.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="17" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>• The material must exist for the selected material type / industry sector.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="17" customHeight="1">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
           <t>• Do not use Update to add a new plant or sales area - use Extend.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>5. GENERAL RULES (ALL TEMPLATES)</t>
         </is>
       </c>
-      <c r="B33" s="4" t="n"/>
-      <c r="C33" s="4" t="n"/>
+      <c r="B32" s="4" t="n"/>
+      <c r="C32" s="4" t="n"/>
+    </row>
+    <row r="33" ht="32" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Data sheet</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>This sheet (Instructions) is for information only. The program reads the DATA sheet, which must be the 2nd sheet of this file. Do not delete, rename or reorder sheets.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="32" customHeight="1">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Data sheet</t>
+          <t>Header rows</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>This sheet (Instructions) is for information only. The program reads the DATA sheet, which must be the 2nd sheet of this file. Do not delete, rename or reorder sheets.</t>
+          <t>Row 3 = technical field names (do not change). Row 4 = field descriptions. Enter data from row 5. Never insert or delete rows 1-4.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="32" customHeight="1">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Header rows</t>
+          <t>One row = one org. level</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Row 3 = technical field names (do not change). Row 4 = field descriptions. Enter data from row 5. Never insert or delete rows 1-4.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="32" customHeight="1">
+          <t>Each row is one plant / storage location / sales area. Repeat the same MATNR (or REFERENCE_MATNR) in several rows to maintain several org. levels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="17" customHeight="1">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>One row = one org. level</t>
+          <t>Column MESSAGE</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Each row is one plant / storage location / sales area. Repeat the same MATNR (or REFERENCE_MATNR) in several rows to maintain several org. levels.</t>
+          <t>Ignored on upload - do not fill. Result messages are shown in the ALV output and result file.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="17" customHeight="1">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>Column MESSAGE</t>
+          <t>Flags X/Y</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Ignored on upload - do not fill. Result messages are shown in the ALV output and result file.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="17" customHeight="1">
+          <t>Switch columns (COPY_..., etc.) accept X, Y, YES, 1 or TRUE. Leave blank for 'no'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="32" customHeight="1">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>Flags X/Y</t>
+          <t>Limits</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Switch columns (COPY_..., etc.) accept X, Y, YES, 1 or TRUE. Leave blank for 'no'.</t>
+          <t>Maximum 1000 rows in foreground. More than 1000 rows: run in BACKGROUND (file on application server). More than 2000 rows: rejected - split the file.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="32" customHeight="1">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>Limits</t>
+          <t>Always test first</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Maximum 1000 rows in foreground. More than 1000 rows: run in BACKGROUND (file on application server). More than 2000 rows: rejected - split the file.</t>
+          <t>Run with 'Test run' ticked, correct all errors, then run again without Test run. Materials with errors are not posted.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="32" customHeight="1">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>Always test first</t>
+          <t>File format</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Run with 'Test run' ticked, correct all errors, then run again without Test run. Materials with errors are not posted.</t>
+          <t>Save as .xlsx (Excel Workbook). No macros, no filters/merged cells in the data area, no formulas - paste values only.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="32" customHeight="1">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>File format</t>
+          <t>Application server</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Save as .xlsx (Excel Workbook). No macros, no filters/merged cells in the data area, no formulas - paste values only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="32" customHeight="1">
-      <c r="A42" s="7" t="inlineStr">
-        <is>
-          <t>Application server</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
           <t>If the file is stored on the application server, copy it in BINARY mode (e.g. CG3Z). ASCII mode damages the xlsx file.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="20">
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B42:C42"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="A29:C29"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A28:C28"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="A31:C31"/>
     <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B37:C37"/>
     <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B37:C37"/>
     <mergeCell ref="A30:C30"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B33:C33"/>
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B41:C41"/>

</xml_diff>